<commit_message>
Update odds files - Mon Sep 14 01:38:39 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
         <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,12 +68,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -435,10 +444,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -499,27 +508,27 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Teoscar Hernandez</t>
+          <t>Pete Alonso</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>+407</t>
+          <t>+321</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>19.7%</t>
+          <t>23.8%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>+407</t>
+          <t>+321</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>19.7%</t>
+          <t>23.8%</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -538,27 +547,27 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Sal Stewart</t>
+          <t>Juan Soto</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>+445</t>
+          <t>+340</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>22.7%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>+445</t>
+          <t>+340</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>22.7%</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -582,22 +591,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>+463</t>
+          <t>+363</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>21.6%</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>+463</t>
+          <t>+363</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>21.6%</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -616,27 +625,27 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Teoscar Hernandez</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>+478</t>
+          <t>+370</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>21.3%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>+478</t>
+          <t>+370</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>21.3%</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -653,68 +662,68 @@
       <c r="I5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Elly De La Cruz</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>+482</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>17.2%</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>+482</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>17.2%</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Coby Mayo</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>+424</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>19.1%</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>+424</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>19.1%</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Enrique Hernandez</t>
+          <t>Francisco Lindor</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>+497</t>
+          <t>+430</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>+497</t>
+          <t>+430</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -733,27 +742,27 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Tyler Stephenson</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>+571</t>
+          <t>+432</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>+571</t>
+          <t>+432</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -772,27 +781,27 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Eugenio Suarez</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>+580</t>
+          <t>+434</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>+580</t>
+          <t>+434</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -809,68 +818,68 @@
       <c r="I9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Tommy Edman</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>+585</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>14.6%</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>+585</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>14.6%</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Christian Encarnacion-Strand</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>+445</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>18.3%</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>+445</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>18.3%</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>JJ Bleday</t>
+          <t>Sal Stewart</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+451</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+451</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -889,27 +898,27 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Vladimir Guerrero Jr.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+464</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>17.7%</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>+620</t>
+          <t>+464</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>17.7%</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -926,68 +935,68 @@
       <c r="I12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Freddie Freeman</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>+630</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>13.7%</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>+630</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>13.7%</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Enrique Hernandez</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>+469</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>17.6%</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>+469</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>17.6%</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Matt McLain</t>
+          <t>George Springer</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+474</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+474</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>12.0%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1006,27 +1015,27 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Josue De Paula</t>
+          <t>Elly De La Cruz</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+487</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>+760</t>
+          <t>+487</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1045,27 +1054,27 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Miguel Rojas</t>
+          <t>Riley Greene</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+499</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+499</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1084,27 +1093,27 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Dane Myers</t>
+          <t>Dylan Beavers</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+508</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>+820</t>
+          <t>+508</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1123,27 +1132,27 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Juan Brito</t>
+          <t>Tommy Edman</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+536</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+536</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1162,27 +1171,27 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Hector Rodriguez</t>
+          <t>Francisco Alvarez</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+538</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+538</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1197,6 +1206,1410 @@
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Gunnar Henderson</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>+560</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>15.2%</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>+560</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>15.2%</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Tyler Stephenson</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>+579</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>+579</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Eugenio Suarez</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>+580</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>+580</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>14.7%</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Brett Baty</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>+587</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>14.6%</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>+587</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>14.6%</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Kyle Tucker</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>+599</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>+599</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Kevin McGonigle</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>JJ Bleday</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Colton Cowser</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Freddie Freeman</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Jared Young</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>+640</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>+640</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Gleyber Torres</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Dillon Dingler</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Narvaez</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>12.7%</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>12.7%</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Matt McLain</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>+730</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>+730</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Bo Bichette</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>11.9%</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>11.9%</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Josue De Paula</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>11.9%</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>11.9%</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Carson Benge</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Alejandro Kirk</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>11.8%</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Miguel Rojas</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>+770</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>+770</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>11.5%</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Heston Kjerstad</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>+810</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>+810</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>AJ Ewing</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Dane Myers</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>+820</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Jackson Holliday</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>+860</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>+860</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Juan Brito</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>+890</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>+890</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>10.1%</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Marcus Semien</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>10.0%</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Josh Smith</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>+910</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>9.9%</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>+910</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>9.9%</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Colt Keith</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>+910</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>9.9%</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>+910</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>9.9%</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Ernie Clement</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>9.7%</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>9.7%</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Nathan Lukes</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>+990</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>9.2%</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>+990</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>9.2%</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Andres Gimenez</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Max Clark</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>+1020</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>+1020</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Brett Callahan</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>+1040</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>+1040</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>8.8%</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Hector Rodriguez</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>+1120</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>8.2%</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>+1120</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>8.2%</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Zach McKinstry</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>+1140</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>+1140</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>John Peck</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>7.7%</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>7.7%</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Brett Bateman</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>+1320</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>7.0%</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>+1320</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>7.0%</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update odds files - Tue Sep 15 21:39:25 UTC 2026
</commit_message>
<xml_diff>
--- a/hr_odds.xlsx
+++ b/hr_odds.xlsx
@@ -1093,27 +1093,27 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Kyle Stowers</t>
+          <t>Munetaka Murakami</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>+356</t>
+          <t>+359</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>21.9%</t>
+          <t>21.8%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>+356</t>
+          <t>+359</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>21.9%</t>
+          <t>21.8%</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1132,27 +1132,27 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Munetaka Murakami</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>+359</t>
+          <t>+360</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>+359</t>
+          <t>+360</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1171,27 +1171,27 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Kazuma Okamoto</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>+360</t>
+          <t>+367</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>21.4%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>+360</t>
+          <t>+367</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>21.4%</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1210,7 +1210,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Kazuma Okamoto</t>
+          <t>Luis Garcia (NYY)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1249,27 +1249,27 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Luis Garcia (NYY)</t>
+          <t>Pete Crow-Armstrong</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>+367</t>
+          <t>+370</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>21.3%</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>+367</t>
+          <t>+370</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>21.3%</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1288,27 +1288,27 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Pete Crow-Armstrong</t>
+          <t>Spencer Jones</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>+370</t>
+          <t>+394</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>21.3%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>+370</t>
+          <t>+394</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>21.3%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1327,12 +1327,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Spencer Jones</t>
+          <t>Ronald Acuna Jr.</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>+394</t>
+          <t>+395</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>+394</t>
+          <t>+395</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1366,27 +1366,27 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Ronald Acuna Jr.</t>
+          <t>Jake Burger</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>+395</t>
+          <t>+397</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>+395</t>
+          <t>+397</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1405,12 +1405,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Jake Burger</t>
+          <t>Kyle Tucker</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>+397</t>
+          <t>+398</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>+397</t>
+          <t>+398</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1444,27 +1444,27 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Kyle Tucker</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>+398</t>
+          <t>+403</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>20.1%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>+398</t>
+          <t>+403</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>20.1%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1483,27 +1483,27 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>+403</t>
+          <t>+405</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>19.8%</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>+403</t>
+          <t>+405</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>19.8%</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1522,27 +1522,27 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>Kyle Stowers</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>+405</t>
+          <t>+407</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>19.7%</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>+405</t>
+          <t>+407</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>19.7%</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1600,7 +1600,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Zach Neto</t>
+          <t>Miguel Vargas</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1639,7 +1639,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Miguel Vargas</t>
+          <t>Zach Neto</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1678,27 +1678,27 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Heriberto Hernandez</t>
+          <t>Ty France</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>+423</t>
+          <t>+425</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>+423</t>
+          <t>+425</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1717,27 +1717,27 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Ty France</t>
+          <t>Eugenio Suarez</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>+425</t>
+          <t>+429</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>+425</t>
+          <t>+429</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1754,92 +1754,92 @@
       <c r="I33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Eugenio Suarez</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>+429</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>18.9%</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>+429</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>18.9%</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr"/>
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Luis Campusano</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>+432</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>18.8%</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>+432</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>18.8%</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr"/>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>Luis Campusano</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>+432</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>18.8%</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>+432</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>18.8%</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr"/>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I35" s="3" t="inlineStr"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Mickey Moniak</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>+434</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>18.7%</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>+434</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>18.7%</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Mickey Moniak</t>
+          <t>Riley Greene</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>+434</t>
+          <t>+436</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>+434</t>
+          <t>+436</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1873,27 +1873,27 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Riley Greene</t>
+          <t>Jose Ramirez</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>+436</t>
+          <t>+437</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>+436</t>
+          <t>+437</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1912,12 +1912,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Jose Ramirez</t>
+          <t>Corey Seager</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>+437</t>
+          <t>+438</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>+437</t>
+          <t>+438</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1990,27 +1990,27 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Corey Seager</t>
+          <t>Alec Burleson</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>+438</t>
+          <t>+443</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.4%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>+438</t>
+          <t>+443</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.4%</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2029,27 +2029,27 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Alec Burleson</t>
+          <t>Randy Arozarena</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>+443</t>
+          <t>+450</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>18.4%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>+443</t>
+          <t>+450</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>18.4%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2107,27 +2107,27 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Randy Arozarena</t>
+          <t>Austin Riley</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+454</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+454</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2146,27 +2146,27 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Austin Riley</t>
+          <t>Freddie Freeman</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>+454</t>
+          <t>+456</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>+454</t>
+          <t>+456</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2183,43 +2183,43 @@
       <c r="I44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Freddie Freeman</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>+456</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>18.0%</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>+456</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>18.0%</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr"/>
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Randal Grichuk</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>+459</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>17.9%</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>+459</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>17.9%</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -2261,43 +2261,43 @@
       <c r="I46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>Randal Grichuk</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>+459</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>17.9%</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>+459</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>17.9%</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr"/>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I47" s="3" t="inlineStr"/>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Heriberto Hernandez</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>+464</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>17.7%</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>+464</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>17.7%</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2339,48 +2339,48 @@
       <c r="I48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Christian Walker</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>+468</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Griffin Conine</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>+467</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
         <is>
           <t>17.6%</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>+468</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>+467</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>17.6%</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr"/>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I49" s="2" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Julio Rodriguez</t>
+          <t>Christian Walker</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -2419,27 +2419,27 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Wilyer Abreu</t>
+          <t>Julio Rodriguez</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>+470</t>
+          <t>+468</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>+470</t>
+          <t>+468</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2458,27 +2458,27 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>JJ Bleday</t>
+          <t>Wilyer Abreu</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>+474</t>
+          <t>+470</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>+474</t>
+          <t>+470</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2536,7 +2536,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Josue De Paula</t>
+          <t>JJ Bleday</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2573,68 +2573,68 @@
       <c r="I54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Rece Hinds</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>+476</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Josue De Paula</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>+474</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
         <is>
           <t>17.4%</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>+476</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>+474</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>17.4%</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr"/>
-      <c r="H55" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I55" s="2" t="inlineStr"/>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr"/>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Willson Contreras</t>
+          <t>Rece Hinds</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+476</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+476</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -2690,68 +2690,68 @@
       <c r="I57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>Sal Stewart</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>+481</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Willson Contreras</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>17.2%</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>+481</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>17.2%</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I58" s="2" t="inlineStr"/>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr"/>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Roman Anthony</t>
+          <t>Sal Stewart</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>+484</t>
+          <t>+481</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>+484</t>
+          <t>+481</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -2770,27 +2770,27 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Michael Harris</t>
+          <t>Roman Anthony</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>+487</t>
+          <t>+484</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>+487</t>
+          <t>+484</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2809,12 +2809,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Jake Bauers</t>
+          <t>Michael Harris</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>+489</t>
+          <t>+487</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2824,7 +2824,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>+489</t>
+          <t>+487</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -2848,27 +2848,27 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Ketel Marte</t>
+          <t>Jake Bauers</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>+490</t>
+          <t>+489</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>+490</t>
+          <t>+489</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -2887,27 +2887,27 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Drake Baldwin</t>
+          <t>Ketel Marte</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>+495</t>
+          <t>+490</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>+495</t>
+          <t>+490</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -2926,12 +2926,12 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Spencer Torkelson</t>
+          <t>Drake Baldwin</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>+497</t>
+          <t>+495</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>+497</t>
+          <t>+495</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -2965,27 +2965,27 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Carter Jensen</t>
+          <t>Spencer Torkelson</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>+498</t>
+          <t>+497</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>+498</t>
+          <t>+497</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -3002,43 +3002,43 @@
       <c r="I65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>Griffin Conine</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>+499</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Carter Jensen</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>+498</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>16.7%</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>+499</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>+498</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>16.7%</t>
         </is>
       </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G66" s="3" t="inlineStr"/>
-      <c r="H66" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I66" s="3" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3160,7 +3160,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Isaac Paredes</t>
+          <t>Heliot Ramos</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -3199,7 +3199,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Heliot Ramos</t>
+          <t>Isaac Paredes</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3236,48 +3236,48 @@
       <c r="I71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>Victor Mesa Jr.</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Corbin Carroll</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>+519</t>
         </is>
       </c>
-      <c r="C72" s="3" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>16.2%</t>
         </is>
       </c>
-      <c r="D72" s="3" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>+519</t>
         </is>
       </c>
-      <c r="E72" s="3" t="inlineStr">
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>16.2%</t>
         </is>
       </c>
-      <c r="F72" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G72" s="3" t="inlineStr"/>
-      <c r="H72" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I72" s="3" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Corbin Carroll</t>
+          <t>Victor Mesa Jr.</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -3750,22 +3750,22 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>+545</t>
+          <t>+550</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>+545</t>
+          <t>+550</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -4174,12 +4174,12 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Michael Busch</t>
+          <t>Royce Lewis</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>+579</t>
+          <t>+578</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -4189,7 +4189,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>+579</t>
+          <t>+578</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -4213,12 +4213,12 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Connor Norby</t>
+          <t>Michael Busch</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>+582</t>
+          <t>+579</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -4228,7 +4228,7 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>+582</t>
+          <t>+579</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -4252,27 +4252,27 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Yandy Diaz</t>
+          <t>Connor Norby</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>+584</t>
+          <t>+582</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>+584</t>
+          <t>+582</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -4291,12 +4291,12 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Jose Siri</t>
+          <t>Yandy Diaz</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>+586</t>
+          <t>+584</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>+586</t>
+          <t>+584</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -4330,27 +4330,27 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Tommy Edman</t>
+          <t>Jose Siri</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>+592</t>
+          <t>+586</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>+592</t>
+          <t>+586</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -4369,27 +4369,27 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Royce Lewis</t>
+          <t>Tommy Edman</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>+593</t>
+          <t>+592</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>+593</t>
+          <t>+592</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
@@ -4445,82 +4445,82 @@
       <c r="I102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="inlineStr">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>Kody Clemens</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G103" s="3" t="inlineStr"/>
+      <c r="H103" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I103" s="3" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
         <is>
           <t>Leonardo Bernal</t>
         </is>
       </c>
-      <c r="B103" s="2" t="inlineStr">
+      <c r="B104" s="2" t="inlineStr">
         <is>
           <t>+600</t>
         </is>
       </c>
-      <c r="C103" s="2" t="inlineStr">
+      <c r="C104" s="2" t="inlineStr">
         <is>
           <t>14.3%</t>
         </is>
       </c>
-      <c r="D103" s="2" t="inlineStr">
+      <c r="D104" s="2" t="inlineStr">
         <is>
           <t>+600</t>
         </is>
       </c>
-      <c r="E103" s="2" t="inlineStr">
+      <c r="E104" s="2" t="inlineStr">
         <is>
           <t>14.3%</t>
         </is>
       </c>
-      <c r="F103" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G103" s="2" t="inlineStr"/>
-      <c r="H103" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I103" s="2" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="3" t="inlineStr">
-        <is>
-          <t>Kody Clemens</t>
-        </is>
-      </c>
-      <c r="B104" s="3" t="inlineStr">
-        <is>
-          <t>+600</t>
-        </is>
-      </c>
-      <c r="C104" s="3" t="inlineStr">
-        <is>
-          <t>14.3%</t>
-        </is>
-      </c>
-      <c r="D104" s="3" t="inlineStr">
-        <is>
-          <t>+600</t>
-        </is>
-      </c>
-      <c r="E104" s="3" t="inlineStr">
-        <is>
-          <t>14.3%</t>
-        </is>
-      </c>
-      <c r="F104" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G104" s="3" t="inlineStr"/>
-      <c r="H104" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I104" s="3" t="inlineStr"/>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -4603,7 +4603,7 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Alex Bregman</t>
+          <t>Jared Young</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -4642,7 +4642,7 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Jared Young</t>
+          <t>Alex Bregman</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Tyrone Taylor</t>
+          <t>Jose Altuve</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -4798,7 +4798,7 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Jose Altuve</t>
+          <t>Tyrone Taylor</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -4876,7 +4876,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Michael Gasper</t>
+          <t>Daulton Varsho</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -4915,7 +4915,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>Daulton Varsho</t>
+          <t>Michael Gasper</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -4954,27 +4954,27 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Tovar</t>
+          <t>Nolan Arenado</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+650</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
@@ -4993,7 +4993,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>Jeremiah Jackson</t>
+          <t>Ezequiel Tovar</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
@@ -5032,7 +5032,7 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Travis Bazzana</t>
+          <t>Jeremiah Jackson</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -5071,7 +5071,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Tim Tawa</t>
+          <t>Travis Bazzana</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -5110,27 +5110,27 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Bryce Eldridge</t>
+          <t>Tim Tawa</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+660</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
@@ -5188,27 +5188,27 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Cedric Mullins</t>
+          <t>Bryce Eldridge</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+670</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
@@ -5227,7 +5227,7 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Anthony Volpe</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -5305,7 +5305,7 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>Anthony Volpe</t>
+          <t>Cedric Mullins</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -5344,27 +5344,27 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>Rafael Flores</t>
+          <t>William Contreras</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+680</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
@@ -5383,7 +5383,7 @@
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>Ozzie Albies</t>
+          <t>Jake Rogers</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
@@ -5422,7 +5422,7 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>Jake Rogers</t>
+          <t>Francisco Alvarez</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -5461,7 +5461,7 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>Yainer Diaz</t>
+          <t>Ozzie Albies</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
@@ -5500,7 +5500,7 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>Francisco Alvarez</t>
+          <t>Yainer Diaz</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -5539,7 +5539,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Nolan Arenado</t>
+          <t>Rafael Flores</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -5578,7 +5578,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>Eduardo Valencia</t>
+          <t>Cole Young</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -5617,7 +5617,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>Marcus Semien</t>
+          <t>Brett Sullivan</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -5656,7 +5656,7 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Pavin Smith</t>
+          <t>Josh Bell</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -5695,7 +5695,7 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Brett Sullivan</t>
+          <t>Eduardo Valencia</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -5734,7 +5734,7 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Cole Young</t>
+          <t>Marcus Semien</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -5773,27 +5773,27 @@
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>Elias Diaz</t>
+          <t>Pavin Smith</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+700</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
@@ -5812,27 +5812,27 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>Ivan Herrera</t>
+          <t>Elias Diaz</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+710</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
@@ -5851,7 +5851,7 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>Andres Chaparro</t>
+          <t>Garrett Mitchell</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
@@ -5890,7 +5890,7 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>Garrett Mitchell</t>
+          <t>Andres Chaparro</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -5929,7 +5929,7 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>Josh Bell</t>
+          <t>Ivan Herrera</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
@@ -5968,7 +5968,7 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>Bryan Reynolds</t>
+          <t>Hunter Feduccia</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -6007,7 +6007,7 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>Hunter Feduccia</t>
+          <t>Bryan Reynolds</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>Carson Kelly</t>
+          <t>Matt McLain</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -6124,7 +6124,7 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>George Lombard Jr.</t>
+          <t>Carson Kelly</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -6163,27 +6163,27 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>Matt McLain</t>
+          <t>Leody Taveras</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+750</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
@@ -6202,7 +6202,7 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>Alec Bohm</t>
+          <t>Dylan Crews</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -6241,7 +6241,7 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>Dylan Crews</t>
+          <t>Carson Benge</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
@@ -6280,7 +6280,7 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>Carson Benge</t>
+          <t>Alec Bohm</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -6319,27 +6319,27 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Leody Taveras</t>
+          <t>Bo Bichette</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+770</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
@@ -6358,7 +6358,7 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>Brady House</t>
+          <t>George Lombard Jr.</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -6436,7 +6436,7 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>Bo Bichette</t>
+          <t>Brady House</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -6475,7 +6475,7 @@
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>Brandon Nimmo</t>
+          <t>Alex Freeland</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -6514,7 +6514,7 @@
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>Alex Freeland</t>
+          <t>Moises Ballesteros</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -6553,7 +6553,7 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>Luis Lara</t>
+          <t>Josh Jung</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -6592,7 +6592,7 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>Josh Jung</t>
+          <t>Brandon Nimmo</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -6631,7 +6631,7 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>Christian Moore</t>
+          <t>Luis Lara</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -6670,7 +6670,7 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>Moises Ballesteros</t>
+          <t>Christian Moore</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
@@ -6709,7 +6709,7 @@
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>Nathan Church</t>
+          <t>Thomas Saggese</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
@@ -6748,7 +6748,7 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Derek Hill</t>
+          <t>Yohel Pozo</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -6787,7 +6787,7 @@
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>Bryan De La Cruz</t>
+          <t>Brenton Doyle</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
@@ -6826,7 +6826,7 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>Thomas Saggese</t>
+          <t>Derek Hill</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -6865,7 +6865,7 @@
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>Yohel Pozo</t>
+          <t>Bryan De La Cruz</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
@@ -6904,7 +6904,7 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>Brenton Doyle</t>
+          <t>Nathan Church</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -6943,7 +6943,7 @@
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>Kyle Karros</t>
+          <t>J.T. Realmuto</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
@@ -6982,7 +6982,7 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>J.T. Realmuto</t>
+          <t>Kyle Karros</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
@@ -7099,7 +7099,7 @@
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>Bryson Stott</t>
+          <t>Hao-Yu Lee</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
@@ -7138,7 +7138,7 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>Carlos Jorge</t>
+          <t>Bryson Stott</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
@@ -7177,7 +7177,7 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>Hao-Yu Lee</t>
+          <t>Carlos Jorge</t>
         </is>
       </c>
       <c r="B173" s="2" t="inlineStr">
@@ -7216,7 +7216,7 @@
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>Angel Genao</t>
+          <t>Jorge Mateo</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -7255,7 +7255,7 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>Jorge Mateo</t>
+          <t>Angel Genao</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -7294,7 +7294,7 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>Otto Lopez</t>
+          <t>Brock Rodden</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -7333,7 +7333,7 @@
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>Brock Rodden</t>
+          <t>Denzer Guzman</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
@@ -7372,27 +7372,27 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>Denzer Guzman</t>
+          <t>Joe Mack</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+860</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
@@ -7450,27 +7450,27 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>Joe Mack</t>
+          <t>Henry Bolte</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>+860</t>
+          <t>+870</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>+860</t>
+          <t>+870</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.3%</t>
         </is>
       </c>
       <c r="F180" s="2" t="inlineStr">
@@ -7489,7 +7489,7 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>Henry Bolte</t>
+          <t>Hector Rodriguez</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
@@ -7528,7 +7528,7 @@
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>Hector Rodriguez</t>
+          <t>AJ Ewing</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
@@ -7567,7 +7567,7 @@
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>AJ Ewing</t>
+          <t>Gabriel Moreno</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
@@ -7606,27 +7606,27 @@
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>Gabriel Moreno</t>
+          <t>Matt Shaw</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>+870</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>+870</t>
+          <t>+880</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="F184" s="2" t="inlineStr">
@@ -7645,27 +7645,27 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>Matt Shaw</t>
+          <t>Michael Massey</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+890</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="F185" s="2" t="inlineStr">
@@ -7684,7 +7684,7 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>Michael Massey</t>
+          <t>Jonah Heim</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
@@ -7723,7 +7723,7 @@
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>Mike Yastrzemski</t>
+          <t>T.J. Rumfield</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
@@ -7762,7 +7762,7 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>Jonah Heim</t>
+          <t>Mike Yastrzemski</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -7801,27 +7801,27 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>T.J. Rumfield</t>
+          <t>Adael Amador</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+900</t>
         </is>
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+900</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="F189" s="2" t="inlineStr">
@@ -7840,7 +7840,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>Ezequiel Duran</t>
+          <t>Brooks Lee</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -7918,7 +7918,7 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>Adael Amador</t>
+          <t>Ezequiel Duran</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -7957,7 +7957,7 @@
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>Brooks Lee</t>
+          <t>Otto Lopez</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
@@ -7996,7 +7996,7 @@
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>Liam Hicks</t>
+          <t>Jordan Lawlar</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
@@ -8035,27 +8035,27 @@
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>Jordan Lawlar</t>
+          <t>Liam Hicks</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+910</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="F195" s="2" t="inlineStr">
@@ -8074,7 +8074,7 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>J.P. Crawford</t>
+          <t>Ali Sanchez</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -8152,7 +8152,7 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>Konnor Griffin</t>
+          <t>J.P. Crawford</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
@@ -8191,27 +8191,27 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>Jonah Cox</t>
+          <t>Konnor Griffin</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+920</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="F199" s="2" t="inlineStr">
@@ -8269,27 +8269,27 @@
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>Richie Palacios</t>
+          <t>Jonah Cox</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+930</t>
         </is>
       </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="F201" s="2" t="inlineStr">
@@ -8308,7 +8308,7 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>Jake McCarthy</t>
+          <t>Jeff McNeil</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -8347,7 +8347,7 @@
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>Jeff McNeil</t>
+          <t>Bryan Torres</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
@@ -8386,7 +8386,7 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>Bryan Torres</t>
+          <t>Richie Palacios</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -8425,7 +8425,7 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>Tristan Peters</t>
+          <t>Jake McCarthy</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -8464,27 +8464,27 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>Osleivis Basabe</t>
+          <t>Tristan Peters</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+940</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="F206" s="2" t="inlineStr">
@@ -8503,7 +8503,7 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>Carlos Cortes</t>
+          <t>Osleivis Basabe</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -8542,7 +8542,7 @@
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>Vaughn Grissom</t>
+          <t>Carlos Cortes</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -8581,27 +8581,27 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Vaughn Grissom</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+950</t>
         </is>
       </c>
       <c r="E209" s="2" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="F209" s="2" t="inlineStr">
@@ -8620,27 +8620,27 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>Jake Cronenworth</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+960</t>
         </is>
       </c>
       <c r="E210" s="2" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="F210" s="2" t="inlineStr">
@@ -8659,7 +8659,7 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>Ali Sanchez</t>
+          <t>Jake Cronenworth</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -8815,7 +8815,7 @@
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>Grant McCray</t>
+          <t>Brice Turang</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -8854,7 +8854,7 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Brice Turang</t>
+          <t>Grant McCray</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -8893,27 +8893,27 @@
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Kaelen Culpepper</t>
+          <t>Emmanuel Rodriguez</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+1000</t>
         </is>
       </c>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="F217" s="2" t="inlineStr">
@@ -8932,7 +8932,7 @@
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Yohandy Morales</t>
+          <t>Donovan Walton</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -9010,7 +9010,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Donovan Walton</t>
+          <t>Yohandy Morales</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -9049,7 +9049,7 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>Brewer Hicklen</t>
+          <t>Kaelen Culpepper</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -9088,27 +9088,27 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>Juan Brito</t>
+          <t>Brewer Hicklen</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1020</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="F222" s="2" t="inlineStr">
@@ -9127,7 +9127,7 @@
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>Emmanuel Rodriguez</t>
+          <t>Sam Antonacci</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -9166,7 +9166,7 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>Sam Antonacci</t>
+          <t>Juan Brito</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -9283,7 +9283,7 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>Caleb Durbin</t>
+          <t>Jakob Marsee</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -9322,7 +9322,7 @@
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>Andres Gimenez</t>
+          <t>Jose Fermin (STL)</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -9361,7 +9361,7 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>Nathan Lukes</t>
+          <t>Caleb Durbin</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -9400,7 +9400,7 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>Jose Fermin (STL)</t>
+          <t>Andres Gimenez</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -9439,27 +9439,27 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>Jakob Marsee</t>
+          <t>Nathan Lukes</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1060</t>
         </is>
       </c>
       <c r="E231" s="2" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="F231" s="2" t="inlineStr">
@@ -9517,7 +9517,7 @@
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>Christian Koss</t>
+          <t>Luke Keaschall</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -9595,7 +9595,7 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>Luke Keaschall</t>
+          <t>Christian Koss</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -9634,7 +9634,7 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>Alika Williams</t>
+          <t>Isaac Collins</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -9673,7 +9673,7 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>Nick Sogard</t>
+          <t>Josh Smith</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -9712,7 +9712,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>Zach McKinstry</t>
+          <t>Luis Arraez</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -9751,7 +9751,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>Josh Smith</t>
+          <t>Zach McKinstry</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -9790,7 +9790,7 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>Isaac Collins</t>
+          <t>Alika Williams</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -9829,7 +9829,7 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>Luis Arraez</t>
+          <t>Nick Sogard</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -9868,7 +9868,7 @@
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>Geraldo Perdomo</t>
+          <t>Brett Bateman</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
@@ -9907,7 +9907,7 @@
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>Brett Bateman</t>
+          <t>Chase Meidroth</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
@@ -9946,7 +9946,7 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>Chase Meidroth</t>
+          <t>Harry Ford</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -9985,7 +9985,7 @@
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>Harry Ford</t>
+          <t>Geraldo Perdomo</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
@@ -10102,27 +10102,27 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>LaMonte Wade Jr.</t>
+          <t>Victor Caratini</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1180</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.8%</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1180</t>
         </is>
       </c>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>7.8%</t>
         </is>
       </c>
       <c r="F248" s="2" t="inlineStr">
@@ -10141,7 +10141,7 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>Victor Caratini</t>
+          <t>Esteury Ruiz</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
@@ -10180,27 +10180,27 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>Ernie Clement</t>
+          <t>LaMonte Wade Jr.</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>+1220</t>
+          <t>+1200</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>7.6%</t>
+          <t>7.7%</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>+1220</t>
+          <t>+1200</t>
         </is>
       </c>
       <c r="E250" s="2" t="inlineStr">
         <is>
-          <t>7.6%</t>
+          <t>7.7%</t>
         </is>
       </c>
       <c r="F250" s="2" t="inlineStr">
@@ -10219,27 +10219,27 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>Nico Hoerner</t>
+          <t>Ernie Clement</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>+1260</t>
+          <t>+1220</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.6%</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
         <is>
-          <t>+1260</t>
+          <t>+1220</t>
         </is>
       </c>
       <c r="E251" s="2" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.6%</t>
         </is>
       </c>
       <c r="F251" s="2" t="inlineStr">
@@ -10258,7 +10258,7 @@
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>Kyle Isbel</t>
+          <t>Nico Hoerner</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
@@ -10297,27 +10297,27 @@
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>Andrew Pinckney</t>
+          <t>Kyle Isbel</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>+1280</t>
+          <t>+1260</t>
         </is>
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.4%</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>+1280</t>
+          <t>+1260</t>
         </is>
       </c>
       <c r="E253" s="2" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.4%</t>
         </is>
       </c>
       <c r="F253" s="2" t="inlineStr">
@@ -10336,7 +10336,7 @@
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>Jacob Young</t>
+          <t>Joey Ortiz</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
@@ -10375,7 +10375,7 @@
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>Javier Sanoja</t>
+          <t>Andrew Pinckney</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
@@ -10414,7 +10414,7 @@
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>Joey Ortiz</t>
+          <t>Jacob Young</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
@@ -10453,7 +10453,7 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>BJ Murray</t>
+          <t>Javier Sanoja</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
@@ -10531,27 +10531,27 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>Esteury Ruiz</t>
+          <t>BJ Murray</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1320</t>
         </is>
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1320</t>
         </is>
       </c>
       <c r="E259" s="2" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="F259" s="2" t="inlineStr">
@@ -10648,7 +10648,7 @@
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>Luisangel Acuna</t>
+          <t>Turner Hill</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
@@ -10687,7 +10687,7 @@
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>Turner Hill</t>
+          <t>Luisangel Acuna</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">

</xml_diff>